<commit_message>
Cenário com peso de 20% para o CSE (três redistribuições)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BauMyZR5unRwjRYRzKjEpf
</commit_message>
<xml_diff>
--- a/metodologia_cidades_inteligentes/resultados/Ranking_Representatividade_original.xlsx
+++ b/metodologia_cidades_inteligentes/resultados/Ranking_Representatividade_original.xlsx
@@ -2538,7 +2538,7 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>0.1403626871885737</v>
+        <v>0.1403626871885736</v>
       </c>
       <c r="M3">
         <v>98</v>
@@ -2582,7 +2582,7 @@
         <v>55</v>
       </c>
       <c r="L4">
-        <v>0.1474928229007858</v>
+        <v>0.1474928229007859</v>
       </c>
       <c r="M4">
         <v>96.7</v>
@@ -2670,7 +2670,7 @@
         <v>98</v>
       </c>
       <c r="L6">
-        <v>0.1496805428184261</v>
+        <v>0.149680542818426</v>
       </c>
       <c r="M6">
         <v>96.3</v>
@@ -2714,7 +2714,7 @@
         <v>58</v>
       </c>
       <c r="L7">
-        <v>0.1510480889393094</v>
+        <v>0.1510480889393095</v>
       </c>
       <c r="M7">
         <v>96.09999999999999</v>
@@ -2758,7 +2758,7 @@
         <v>38</v>
       </c>
       <c r="L8">
-        <v>0.1524535807715782</v>
+        <v>0.1524535807715783</v>
       </c>
       <c r="M8">
         <v>95.90000000000001</v>
@@ -2934,7 +2934,7 @@
         <v>66</v>
       </c>
       <c r="L12">
-        <v>0.1617839338873964</v>
+        <v>0.1617839338873965</v>
       </c>
       <c r="M12">
         <v>94.2</v>
@@ -3154,7 +3154,7 @@
         <v>47</v>
       </c>
       <c r="L17">
-        <v>0.1698161970669634</v>
+        <v>0.1698161970669635</v>
       </c>
       <c r="M17">
         <v>92.8</v>
@@ -3198,7 +3198,7 @@
         <v>85</v>
       </c>
       <c r="L18">
-        <v>0.1702662460483715</v>
+        <v>0.1702662460483714</v>
       </c>
       <c r="M18">
         <v>92.7</v>
@@ -3330,7 +3330,7 @@
         <v>48</v>
       </c>
       <c r="L21">
-        <v>0.1731922928098998</v>
+        <v>0.1731922928098999</v>
       </c>
       <c r="M21">
         <v>92.2</v>
@@ -3506,7 +3506,7 @@
         <v>76</v>
       </c>
       <c r="L25">
-        <v>0.1838133232051724</v>
+        <v>0.1838133232051725</v>
       </c>
       <c r="M25">
         <v>90.40000000000001</v>
@@ -3638,7 +3638,7 @@
         <v>73</v>
       </c>
       <c r="L28">
-        <v>0.1866544826352131</v>
+        <v>0.186654482635213</v>
       </c>
       <c r="M28">
         <v>89.90000000000001</v>
@@ -3726,7 +3726,7 @@
         <v>45</v>
       </c>
       <c r="L30">
-        <v>0.1959567404147378</v>
+        <v>0.1959567404147379</v>
       </c>
       <c r="M30">
         <v>88.2</v>
@@ -3902,7 +3902,7 @@
         <v>30</v>
       </c>
       <c r="L34">
-        <v>0.2001129038702077</v>
+        <v>0.2001129038702078</v>
       </c>
       <c r="M34">
         <v>87.5</v>
@@ -3990,7 +3990,7 @@
         <v>114</v>
       </c>
       <c r="L36">
-        <v>0.2046426436845739</v>
+        <v>0.2046426436845738</v>
       </c>
       <c r="M36">
         <v>86.7</v>
@@ -4298,7 +4298,7 @@
         <v>82</v>
       </c>
       <c r="L43">
-        <v>0.2178912018296183</v>
+        <v>0.2178912018296184</v>
       </c>
       <c r="M43">
         <v>84.40000000000001</v>
@@ -4386,7 +4386,7 @@
         <v>75</v>
       </c>
       <c r="L45">
-        <v>0.2249637522833901</v>
+        <v>0.2249637522833902</v>
       </c>
       <c r="M45">
         <v>83.2</v>
@@ -4430,7 +4430,7 @@
         <v>84</v>
       </c>
       <c r="L46">
-        <v>0.225905559330795</v>
+        <v>0.2259055593307951</v>
       </c>
       <c r="M46">
         <v>83</v>
@@ -5266,7 +5266,7 @@
         <v>56</v>
       </c>
       <c r="L65">
-        <v>0.2815479934793909</v>
+        <v>0.2815479934793908</v>
       </c>
       <c r="M65">
         <v>73.3</v>
@@ -5310,7 +5310,7 @@
         <v>42</v>
       </c>
       <c r="L66">
-        <v>0.2898061314442719</v>
+        <v>0.2898061314442718</v>
       </c>
       <c r="M66">
         <v>71.8</v>
@@ -5354,7 +5354,7 @@
         <v>129</v>
       </c>
       <c r="L67">
-        <v>0.2918151173914641</v>
+        <v>0.291815117391464</v>
       </c>
       <c r="M67">
         <v>71.5</v>
@@ -5530,7 +5530,7 @@
         <v>34</v>
       </c>
       <c r="L71">
-        <v>0.3062677394673963</v>
+        <v>0.3062677394673964</v>
       </c>
       <c r="M71">
         <v>69</v>
@@ -5882,7 +5882,7 @@
         <v>133</v>
       </c>
       <c r="L79">
-        <v>0.3228086422382559</v>
+        <v>0.3228086422382558</v>
       </c>
       <c r="M79">
         <v>66.09999999999999</v>
@@ -6102,7 +6102,7 @@
         <v>134</v>
       </c>
       <c r="L84">
-        <v>0.3325754471893058</v>
+        <v>0.3325754471893057</v>
       </c>
       <c r="M84">
         <v>64.40000000000001</v>
@@ -6146,7 +6146,7 @@
         <v>138</v>
       </c>
       <c r="L85">
-        <v>0.3347845326182452</v>
+        <v>0.3347845326182451</v>
       </c>
       <c r="M85">
         <v>64</v>
@@ -6410,7 +6410,7 @@
         <v>14</v>
       </c>
       <c r="L91">
-        <v>0.3458896633215852</v>
+        <v>0.3458896633215853</v>
       </c>
       <c r="M91">
         <v>62</v>
@@ -6542,7 +6542,7 @@
         <v>23</v>
       </c>
       <c r="L94">
-        <v>0.3574547831687518</v>
+        <v>0.3574547831687519</v>
       </c>
       <c r="M94">
         <v>60</v>
@@ -6674,7 +6674,7 @@
         <v>77</v>
       </c>
       <c r="L97">
-        <v>0.3736830214511383</v>
+        <v>0.3736830214511384</v>
       </c>
       <c r="M97">
         <v>57.2</v>
@@ -6718,7 +6718,7 @@
         <v>93</v>
       </c>
       <c r="L98">
-        <v>0.3810698345330376</v>
+        <v>0.3810698345330375</v>
       </c>
       <c r="M98">
         <v>55.9</v>
@@ -6850,7 +6850,7 @@
         <v>135</v>
       </c>
       <c r="L101">
-        <v>0.387560810637252</v>
+        <v>0.3875608106372519</v>
       </c>
       <c r="M101">
         <v>54.8</v>
@@ -7026,7 +7026,7 @@
         <v>140</v>
       </c>
       <c r="L105">
-        <v>0.4051650391163914</v>
+        <v>0.4051650391163913</v>
       </c>
       <c r="M105">
         <v>51.7</v>
@@ -7114,7 +7114,7 @@
         <v>106</v>
       </c>
       <c r="L107">
-        <v>0.41031742447693</v>
+        <v>0.4103174244769299</v>
       </c>
       <c r="M107">
         <v>50.8</v>
@@ -8610,7 +8610,7 @@
         <v>5</v>
       </c>
       <c r="L141">
-        <v>0.6137238982075762</v>
+        <v>0.6137238982075763</v>
       </c>
       <c r="M141">
         <v>15.2</v>
@@ -8698,7 +8698,7 @@
         <v>26</v>
       </c>
       <c r="L143">
-        <v>0.6362015682019516</v>
+        <v>0.6362015682019517</v>
       </c>
       <c r="M143">
         <v>11.3</v>
@@ -8874,7 +8874,7 @@
         <v>115</v>
       </c>
       <c r="L147">
-        <v>0.06619144333400193</v>
+        <v>0.06619144333400194</v>
       </c>
       <c r="M147">
         <v>100</v>
@@ -8918,7 +8918,7 @@
         <v>136</v>
       </c>
       <c r="L148">
-        <v>0.06715442762708859</v>
+        <v>0.06715442762708856</v>
       </c>
       <c r="M148">
         <v>99.90000000000001</v>
@@ -8962,7 +8962,7 @@
         <v>127</v>
       </c>
       <c r="L149">
-        <v>0.07029108843014432</v>
+        <v>0.07029108843014437</v>
       </c>
       <c r="M149">
         <v>99.5</v>
@@ -9006,7 +9006,7 @@
         <v>107</v>
       </c>
       <c r="L150">
-        <v>0.07091316139324405</v>
+        <v>0.07091316139324408</v>
       </c>
       <c r="M150">
         <v>99.40000000000001</v>
@@ -9050,7 +9050,7 @@
         <v>109</v>
       </c>
       <c r="L151">
-        <v>0.07248601494447167</v>
+        <v>0.07248601494447171</v>
       </c>
       <c r="M151">
         <v>99.2</v>
@@ -9094,7 +9094,7 @@
         <v>123</v>
       </c>
       <c r="L152">
-        <v>0.07954104871917982</v>
+        <v>0.07954104871917984</v>
       </c>
       <c r="M152">
         <v>98.3</v>
@@ -9138,7 +9138,7 @@
         <v>142</v>
       </c>
       <c r="L153">
-        <v>0.08345345886506302</v>
+        <v>0.08345345886506304</v>
       </c>
       <c r="M153">
         <v>97.8</v>
@@ -9182,7 +9182,7 @@
         <v>147</v>
       </c>
       <c r="L154">
-        <v>0.0852218380005603</v>
+        <v>0.08522183800056025</v>
       </c>
       <c r="M154">
         <v>97.5</v>
@@ -9226,7 +9226,7 @@
         <v>103</v>
       </c>
       <c r="L155">
-        <v>0.08807377044332071</v>
+        <v>0.08807377044332075</v>
       </c>
       <c r="M155">
         <v>97.2</v>
@@ -9270,7 +9270,7 @@
         <v>94</v>
       </c>
       <c r="L156">
-        <v>0.08825008735098548</v>
+        <v>0.08825008735098551</v>
       </c>
       <c r="M156">
         <v>97.2</v>
@@ -9314,7 +9314,7 @@
         <v>130</v>
       </c>
       <c r="L157">
-        <v>0.08853929308511348</v>
+        <v>0.0885392930851135</v>
       </c>
       <c r="M157">
         <v>97.09999999999999</v>
@@ -9402,7 +9402,7 @@
         <v>93</v>
       </c>
       <c r="L159">
-        <v>0.09446266645596996</v>
+        <v>0.0944626664559699</v>
       </c>
       <c r="M159">
         <v>96.40000000000001</v>
@@ -9446,7 +9446,7 @@
         <v>95</v>
       </c>
       <c r="L160">
-        <v>0.09460288533901229</v>
+        <v>0.09460288533901234</v>
       </c>
       <c r="M160">
         <v>96.3</v>
@@ -9490,7 +9490,7 @@
         <v>104</v>
       </c>
       <c r="L161">
-        <v>0.09945727491143193</v>
+        <v>0.09945727491143191</v>
       </c>
       <c r="M161">
         <v>95.7</v>
@@ -9534,7 +9534,7 @@
         <v>96</v>
       </c>
       <c r="L162">
-        <v>0.1003661397289795</v>
+        <v>0.1003661397289796</v>
       </c>
       <c r="M162">
         <v>95.59999999999999</v>
@@ -9578,7 +9578,7 @@
         <v>87</v>
       </c>
       <c r="L163">
-        <v>0.1015534551501083</v>
+        <v>0.1015534551501084</v>
       </c>
       <c r="M163">
         <v>95.40000000000001</v>
@@ -9622,7 +9622,7 @@
         <v>137</v>
       </c>
       <c r="L164">
-        <v>0.1072228769104766</v>
+        <v>0.1072228769104765</v>
       </c>
       <c r="M164">
         <v>94.7</v>
@@ -9930,7 +9930,7 @@
         <v>74</v>
       </c>
       <c r="L171">
-        <v>0.1141725707738877</v>
+        <v>0.1141725707738878</v>
       </c>
       <c r="M171">
         <v>93.8</v>
@@ -9974,7 +9974,7 @@
         <v>164</v>
       </c>
       <c r="L172">
-        <v>0.1157274392700837</v>
+        <v>0.1157274392700836</v>
       </c>
       <c r="M172">
         <v>93.59999999999999</v>
@@ -10106,7 +10106,7 @@
         <v>92</v>
       </c>
       <c r="L175">
-        <v>0.1191362439243541</v>
+        <v>0.1191362439243542</v>
       </c>
       <c r="M175">
         <v>93.2</v>
@@ -10150,7 +10150,7 @@
         <v>80</v>
       </c>
       <c r="L176">
-        <v>0.1204865351368388</v>
+        <v>0.1204865351368389</v>
       </c>
       <c r="M176">
         <v>93</v>
@@ -10502,7 +10502,7 @@
         <v>78</v>
       </c>
       <c r="L184">
-        <v>0.140310371877768</v>
+        <v>0.1403103718777681</v>
       </c>
       <c r="M184">
         <v>90.40000000000001</v>
@@ -10546,7 +10546,7 @@
         <v>157</v>
       </c>
       <c r="L185">
-        <v>0.1491389092853659</v>
+        <v>0.1491389092853658</v>
       </c>
       <c r="M185">
         <v>89.3</v>
@@ -10590,7 +10590,7 @@
         <v>81</v>
       </c>
       <c r="L186">
-        <v>0.1494215782095936</v>
+        <v>0.1494215782095937</v>
       </c>
       <c r="M186">
         <v>89.3</v>
@@ -10722,7 +10722,7 @@
         <v>77</v>
       </c>
       <c r="L189">
-        <v>0.1551230661247232</v>
+        <v>0.1551230661247233</v>
       </c>
       <c r="M189">
         <v>88.5</v>
@@ -11206,7 +11206,7 @@
         <v>134</v>
       </c>
       <c r="L200">
-        <v>0.1761652202675335</v>
+        <v>0.1761652202675336</v>
       </c>
       <c r="M200">
         <v>85.8</v>
@@ -11470,7 +11470,7 @@
         <v>106</v>
       </c>
       <c r="L206">
-        <v>0.1864245252343707</v>
+        <v>0.1864245252343708</v>
       </c>
       <c r="M206">
         <v>84.5</v>
@@ -11514,7 +11514,7 @@
         <v>192</v>
       </c>
       <c r="L207">
-        <v>0.1883221711736665</v>
+        <v>0.1883221711736664</v>
       </c>
       <c r="M207">
         <v>84.2</v>
@@ -11822,7 +11822,7 @@
         <v>91</v>
       </c>
       <c r="L214">
-        <v>0.2051476402282762</v>
+        <v>0.2051476402282761</v>
       </c>
       <c r="M214">
         <v>82.09999999999999</v>
@@ -11954,7 +11954,7 @@
         <v>207</v>
       </c>
       <c r="L217">
-        <v>0.2101380007244849</v>
+        <v>0.2101380007244848</v>
       </c>
       <c r="M217">
         <v>81.40000000000001</v>
@@ -12086,7 +12086,7 @@
         <v>208</v>
       </c>
       <c r="L220">
-        <v>0.2129301428057815</v>
+        <v>0.2129301428057814</v>
       </c>
       <c r="M220">
         <v>81.09999999999999</v>
@@ -12262,7 +12262,7 @@
         <v>202</v>
       </c>
       <c r="L224">
-        <v>0.2174163731268174</v>
+        <v>0.2174163731268173</v>
       </c>
       <c r="M224">
         <v>80.5</v>
@@ -12350,7 +12350,7 @@
         <v>159</v>
       </c>
       <c r="L226">
-        <v>0.2189888690963271</v>
+        <v>0.2189888690963272</v>
       </c>
       <c r="M226">
         <v>80.3</v>
@@ -12394,7 +12394,7 @@
         <v>88</v>
       </c>
       <c r="L227">
-        <v>0.2205382870443673</v>
+        <v>0.2205382870443672</v>
       </c>
       <c r="M227">
         <v>80.09999999999999</v>
@@ -12482,7 +12482,7 @@
         <v>196</v>
       </c>
       <c r="L229">
-        <v>0.2218980343320819</v>
+        <v>0.2218980343320818</v>
       </c>
       <c r="M229">
         <v>79.90000000000001</v>
@@ -12658,7 +12658,7 @@
         <v>186</v>
       </c>
       <c r="L233">
-        <v>0.2246721413402896</v>
+        <v>0.2246721413402895</v>
       </c>
       <c r="M233">
         <v>79.5</v>
@@ -12702,7 +12702,7 @@
         <v>201</v>
       </c>
       <c r="L234">
-        <v>0.2267441572441863</v>
+        <v>0.2267441572441862</v>
       </c>
       <c r="M234">
         <v>79.3</v>
@@ -12834,7 +12834,7 @@
         <v>158</v>
       </c>
       <c r="L237">
-        <v>0.2311988586407836</v>
+        <v>0.2311988586407835</v>
       </c>
       <c r="M237">
         <v>78.7</v>
@@ -12922,7 +12922,7 @@
         <v>210</v>
       </c>
       <c r="L239">
-        <v>0.2334149594409634</v>
+        <v>0.2334149594409633</v>
       </c>
       <c r="M239">
         <v>78.40000000000001</v>
@@ -13054,7 +13054,7 @@
         <v>180</v>
       </c>
       <c r="L242">
-        <v>0.2410977846544468</v>
+        <v>0.2410977846544469</v>
       </c>
       <c r="M242">
         <v>77.40000000000001</v>
@@ -13230,7 +13230,7 @@
         <v>90</v>
       </c>
       <c r="L246">
-        <v>0.244488835111269</v>
+        <v>0.2444888351112691</v>
       </c>
       <c r="M246">
         <v>77</v>
@@ -13274,7 +13274,7 @@
         <v>214</v>
       </c>
       <c r="L247">
-        <v>0.2466889483906994</v>
+        <v>0.2466889483906993</v>
       </c>
       <c r="M247">
         <v>76.7</v>
@@ -13494,7 +13494,7 @@
         <v>173</v>
       </c>
       <c r="L252">
-        <v>0.2509227918148113</v>
+        <v>0.2509227918148112</v>
       </c>
       <c r="M252">
         <v>76.2</v>
@@ -13538,7 +13538,7 @@
         <v>219</v>
       </c>
       <c r="L253">
-        <v>0.2519182810745849</v>
+        <v>0.2519182810745848</v>
       </c>
       <c r="M253">
         <v>76</v>
@@ -13626,7 +13626,7 @@
         <v>206</v>
       </c>
       <c r="L255">
-        <v>0.2533634259137674</v>
+        <v>0.2533634259137673</v>
       </c>
       <c r="M255">
         <v>75.8</v>
@@ -13978,7 +13978,7 @@
         <v>195</v>
       </c>
       <c r="L263">
-        <v>0.2699909280914295</v>
+        <v>0.2699909280914294</v>
       </c>
       <c r="M263">
         <v>73.7</v>
@@ -14066,7 +14066,7 @@
         <v>133</v>
       </c>
       <c r="L265">
-        <v>0.2725843561618672</v>
+        <v>0.2725843561618673</v>
       </c>
       <c r="M265">
         <v>73.40000000000001</v>
@@ -14154,7 +14154,7 @@
         <v>163</v>
       </c>
       <c r="L267">
-        <v>0.2728322124303684</v>
+        <v>0.2728322124303685</v>
       </c>
       <c r="M267">
         <v>73.3</v>
@@ -14286,7 +14286,7 @@
         <v>216</v>
       </c>
       <c r="L270">
-        <v>0.2757492352233143</v>
+        <v>0.2757492352233142</v>
       </c>
       <c r="M270">
         <v>72.90000000000001</v>
@@ -14374,7 +14374,7 @@
         <v>119</v>
       </c>
       <c r="L272">
-        <v>0.2770556573172419</v>
+        <v>0.2770556573172418</v>
       </c>
       <c r="M272">
         <v>72.8</v>
@@ -14418,7 +14418,7 @@
         <v>222</v>
       </c>
       <c r="L273">
-        <v>0.2807825860136882</v>
+        <v>0.2807825860136881</v>
       </c>
       <c r="M273">
         <v>72.3</v>
@@ -14550,7 +14550,7 @@
         <v>167</v>
       </c>
       <c r="L276">
-        <v>0.2880326716354359</v>
+        <v>0.2880326716354358</v>
       </c>
       <c r="M276">
         <v>71.40000000000001</v>
@@ -14594,7 +14594,7 @@
         <v>48</v>
       </c>
       <c r="L277">
-        <v>0.2916828093806095</v>
+        <v>0.2916828093806094</v>
       </c>
       <c r="M277">
         <v>70.90000000000001</v>
@@ -14638,7 +14638,7 @@
         <v>53</v>
       </c>
       <c r="L278">
-        <v>0.2920206248202434</v>
+        <v>0.2920206248202433</v>
       </c>
       <c r="M278">
         <v>70.8</v>
@@ -14726,7 +14726,7 @@
         <v>143</v>
       </c>
       <c r="L280">
-        <v>0.2934319279821763</v>
+        <v>0.2934319279821762</v>
       </c>
       <c r="M280">
         <v>70.7</v>
@@ -14902,7 +14902,7 @@
         <v>66</v>
       </c>
       <c r="L284">
-        <v>0.3052899305347767</v>
+        <v>0.3052899305347766</v>
       </c>
       <c r="M284">
         <v>69.09999999999999</v>
@@ -14990,7 +14990,7 @@
         <v>111</v>
       </c>
       <c r="L286">
-        <v>0.3155071473908811</v>
+        <v>0.315507147390881</v>
       </c>
       <c r="M286">
         <v>67.8</v>
@@ -15122,7 +15122,7 @@
         <v>179</v>
       </c>
       <c r="L289">
-        <v>0.3198205282242169</v>
+        <v>0.3198205282242168</v>
       </c>
       <c r="M289">
         <v>67.3</v>
@@ -15342,7 +15342,7 @@
         <v>54</v>
       </c>
       <c r="L294">
-        <v>0.3249300004051161</v>
+        <v>0.3249300004051162</v>
       </c>
       <c r="M294">
         <v>66.59999999999999</v>
@@ -15606,7 +15606,7 @@
         <v>228</v>
       </c>
       <c r="L300">
-        <v>0.3348204414266723</v>
+        <v>0.3348204414266722</v>
       </c>
       <c r="M300">
         <v>65.3</v>
@@ -15694,7 +15694,7 @@
         <v>213</v>
       </c>
       <c r="L302">
-        <v>0.3357581096364126</v>
+        <v>0.3357581096364125</v>
       </c>
       <c r="M302">
         <v>65.2</v>
@@ -15738,7 +15738,7 @@
         <v>189</v>
       </c>
       <c r="L303">
-        <v>0.3367468335630793</v>
+        <v>0.3367468335630792</v>
       </c>
       <c r="M303">
         <v>65.09999999999999</v>
@@ -15958,7 +15958,7 @@
         <v>15</v>
       </c>
       <c r="L308">
-        <v>0.3508230197909936</v>
+        <v>0.3508230197909937</v>
       </c>
       <c r="M308">
         <v>63.3</v>
@@ -16002,7 +16002,7 @@
         <v>34</v>
       </c>
       <c r="L309">
-        <v>0.3509011557691879</v>
+        <v>0.350901155769188</v>
       </c>
       <c r="M309">
         <v>63.2</v>
@@ -16090,7 +16090,7 @@
         <v>199</v>
       </c>
       <c r="L311">
-        <v>0.3522516630892125</v>
+        <v>0.3522516630892124</v>
       </c>
       <c r="M311">
         <v>63.1</v>
@@ -16266,7 +16266,7 @@
         <v>233</v>
       </c>
       <c r="L315">
-        <v>0.3609800144881061</v>
+        <v>0.360980014488106</v>
       </c>
       <c r="M315">
         <v>61.9</v>
@@ -16398,7 +16398,7 @@
         <v>170</v>
       </c>
       <c r="L318">
-        <v>0.3683041266994669</v>
+        <v>0.3683041266994668</v>
       </c>
       <c r="M318">
         <v>61</v>
@@ -16486,7 +16486,7 @@
         <v>220</v>
       </c>
       <c r="L320">
-        <v>0.3711839179790558</v>
+        <v>0.3711839179790557</v>
       </c>
       <c r="M320">
         <v>60.6</v>
@@ -16530,7 +16530,7 @@
         <v>9</v>
       </c>
       <c r="L321">
-        <v>0.3732321301602673</v>
+        <v>0.3732321301602674</v>
       </c>
       <c r="M321">
         <v>60.4</v>
@@ -16574,7 +16574,7 @@
         <v>128</v>
       </c>
       <c r="L322">
-        <v>0.3747764600396702</v>
+        <v>0.3747764600396703</v>
       </c>
       <c r="M322">
         <v>60.2</v>
@@ -16662,7 +16662,7 @@
         <v>234</v>
       </c>
       <c r="L324">
-        <v>0.3803624720333128</v>
+        <v>0.3803624720333127</v>
       </c>
       <c r="M324">
         <v>59.4</v>
@@ -16706,7 +16706,7 @@
         <v>30</v>
       </c>
       <c r="L325">
-        <v>0.3810451017779291</v>
+        <v>0.3810451017779292</v>
       </c>
       <c r="M325">
         <v>59.4</v>
@@ -16750,7 +16750,7 @@
         <v>237</v>
       </c>
       <c r="L326">
-        <v>0.3825584156039315</v>
+        <v>0.3825584156039314</v>
       </c>
       <c r="M326">
         <v>59.2</v>
@@ -16838,7 +16838,7 @@
         <v>29</v>
       </c>
       <c r="L328">
-        <v>0.3827519435840236</v>
+        <v>0.3827519435840237</v>
       </c>
       <c r="M328">
         <v>59.1</v>
@@ -17190,7 +17190,7 @@
         <v>25</v>
       </c>
       <c r="L336">
-        <v>0.4011946231080378</v>
+        <v>0.4011946231080379</v>
       </c>
       <c r="M336">
         <v>56.8</v>
@@ -17322,7 +17322,7 @@
         <v>231</v>
       </c>
       <c r="L339">
-        <v>0.4098824757247638</v>
+        <v>0.4098824757247637</v>
       </c>
       <c r="M339">
         <v>55.6</v>
@@ -17366,7 +17366,7 @@
         <v>28</v>
       </c>
       <c r="L340">
-        <v>0.4108438235001471</v>
+        <v>0.4108438235001472</v>
       </c>
       <c r="M340">
         <v>55.5</v>
@@ -17410,7 +17410,7 @@
         <v>24</v>
       </c>
       <c r="L341">
-        <v>0.414848161792429</v>
+        <v>0.4148481617924291</v>
       </c>
       <c r="M341">
         <v>55</v>
@@ -17454,7 +17454,7 @@
         <v>239</v>
       </c>
       <c r="L342">
-        <v>0.4151358463026983</v>
+        <v>0.4151358463026982</v>
       </c>
       <c r="M342">
         <v>55</v>
@@ -17542,7 +17542,7 @@
         <v>118</v>
       </c>
       <c r="L344">
-        <v>0.4182731442488799</v>
+        <v>0.41827314424888</v>
       </c>
       <c r="M344">
         <v>54.5</v>
@@ -17938,7 +17938,7 @@
         <v>168</v>
       </c>
       <c r="L353">
-        <v>0.445023479997479</v>
+        <v>0.4450234799974789</v>
       </c>
       <c r="M353">
         <v>51.1</v>
@@ -18070,7 +18070,7 @@
         <v>120</v>
       </c>
       <c r="L356">
-        <v>0.4511004045387178</v>
+        <v>0.4511004045387179</v>
       </c>
       <c r="M356">
         <v>50.3</v>
@@ -18114,7 +18114,7 @@
         <v>14</v>
       </c>
       <c r="L357">
-        <v>0.451393682063099</v>
+        <v>0.4513936820630991</v>
       </c>
       <c r="M357">
         <v>50.3</v>
@@ -18202,7 +18202,7 @@
         <v>101</v>
       </c>
       <c r="L359">
-        <v>0.4574999081816309</v>
+        <v>0.4574999081816308</v>
       </c>
       <c r="M359">
         <v>49.5</v>
@@ -18598,7 +18598,7 @@
         <v>39</v>
       </c>
       <c r="L368">
-        <v>0.5013384441577097</v>
+        <v>0.5013384441577098</v>
       </c>
       <c r="M368">
         <v>43.8</v>
@@ -18686,7 +18686,7 @@
         <v>131</v>
       </c>
       <c r="L370">
-        <v>0.5052843375385817</v>
+        <v>0.5052843375385816</v>
       </c>
       <c r="M370">
         <v>43.3</v>
@@ -18774,7 +18774,7 @@
         <v>8</v>
       </c>
       <c r="L372">
-        <v>0.5145246249870303</v>
+        <v>0.5145246249870304</v>
       </c>
       <c r="M372">
         <v>42.1</v>
@@ -18862,7 +18862,7 @@
         <v>12</v>
       </c>
       <c r="L374">
-        <v>0.5326721585228572</v>
+        <v>0.5326721585228573</v>
       </c>
       <c r="M374">
         <v>39.8</v>
@@ -18950,7 +18950,7 @@
         <v>205</v>
       </c>
       <c r="L376">
-        <v>0.5466190276897037</v>
+        <v>0.5466190276897036</v>
       </c>
       <c r="M376">
         <v>38</v>
@@ -19214,7 +19214,7 @@
         <v>72</v>
       </c>
       <c r="L382">
-        <v>0.6190479288792963</v>
+        <v>0.6190479288792962</v>
       </c>
       <c r="M382">
         <v>28.6</v>
@@ -19346,7 +19346,7 @@
         <v>2</v>
       </c>
       <c r="L385">
-        <v>0.6737571842097811</v>
+        <v>0.6737571842097813</v>
       </c>
       <c r="M385">
         <v>21.6</v>
@@ -27398,7 +27398,7 @@
         <v>28</v>
       </c>
       <c r="L568">
-        <v>0.07128055890117352</v>
+        <v>0.0712805589011736</v>
       </c>
       <c r="M568">
         <v>100</v>
@@ -27442,7 +27442,7 @@
         <v>26</v>
       </c>
       <c r="L569">
-        <v>0.07792670351053872</v>
+        <v>0.07792670351053879</v>
       </c>
       <c r="M569">
         <v>99.40000000000001</v>
@@ -27530,7 +27530,7 @@
         <v>39</v>
       </c>
       <c r="L571">
-        <v>0.1674395219602271</v>
+        <v>0.1674395219602272</v>
       </c>
       <c r="M571">
         <v>91.5</v>
@@ -27838,7 +27838,7 @@
         <v>54</v>
       </c>
       <c r="L578">
-        <v>0.2904114250516914</v>
+        <v>0.2904114250516913</v>
       </c>
       <c r="M578">
         <v>80.7</v>
@@ -27882,7 +27882,7 @@
         <v>18</v>
       </c>
       <c r="L579">
-        <v>0.2913713974899776</v>
+        <v>0.2913713974899777</v>
       </c>
       <c r="M579">
         <v>80.59999999999999</v>
@@ -27926,7 +27926,7 @@
         <v>49</v>
       </c>
       <c r="L580">
-        <v>0.3027357065327597</v>
+        <v>0.3027357065327598</v>
       </c>
       <c r="M580">
         <v>79.59999999999999</v>
@@ -28014,7 +28014,7 @@
         <v>41</v>
       </c>
       <c r="L582">
-        <v>0.3100698640009279</v>
+        <v>0.3100698640009278</v>
       </c>
       <c r="M582">
         <v>79</v>
@@ -28102,7 +28102,7 @@
         <v>67</v>
       </c>
       <c r="L584">
-        <v>0.3267416560114995</v>
+        <v>0.3267416560114994</v>
       </c>
       <c r="M584">
         <v>77.5</v>
@@ -28146,7 +28146,7 @@
         <v>50</v>
       </c>
       <c r="L585">
-        <v>0.3290873523961549</v>
+        <v>0.3290873523961547</v>
       </c>
       <c r="M585">
         <v>77.3</v>
@@ -28234,7 +28234,7 @@
         <v>65</v>
       </c>
       <c r="L587">
-        <v>0.347393550257404</v>
+        <v>0.3473935502574039</v>
       </c>
       <c r="M587">
         <v>75.7</v>
@@ -28322,7 +28322,7 @@
         <v>55</v>
       </c>
       <c r="L589">
-        <v>0.3535506957768254</v>
+        <v>0.3535506957768253</v>
       </c>
       <c r="M589">
         <v>75.2</v>
@@ -28366,7 +28366,7 @@
         <v>56</v>
       </c>
       <c r="L590">
-        <v>0.3600992687924484</v>
+        <v>0.3600992687924483</v>
       </c>
       <c r="M590">
         <v>74.59999999999999</v>
@@ -28410,7 +28410,7 @@
         <v>58</v>
       </c>
       <c r="L591">
-        <v>0.3602971924740764</v>
+        <v>0.3602971924740763</v>
       </c>
       <c r="M591">
         <v>74.59999999999999</v>
@@ -28454,7 +28454,7 @@
         <v>52</v>
       </c>
       <c r="L592">
-        <v>0.361497987079296</v>
+        <v>0.3614979870792959</v>
       </c>
       <c r="M592">
         <v>74.5</v>
@@ -28498,7 +28498,7 @@
         <v>62</v>
       </c>
       <c r="L593">
-        <v>0.3655465856744913</v>
+        <v>0.3655465856744912</v>
       </c>
       <c r="M593">
         <v>74.09999999999999</v>
@@ -28586,7 +28586,7 @@
         <v>45</v>
       </c>
       <c r="L595">
-        <v>0.3760626143654405</v>
+        <v>0.3760626143654404</v>
       </c>
       <c r="M595">
         <v>73.2</v>
@@ -28630,7 +28630,7 @@
         <v>53</v>
       </c>
       <c r="L596">
-        <v>0.3766402829386803</v>
+        <v>0.3766402829386802</v>
       </c>
       <c r="M596">
         <v>73.09999999999999</v>
@@ -28762,7 +28762,7 @@
         <v>36</v>
       </c>
       <c r="L599">
-        <v>0.3858858495747154</v>
+        <v>0.3858858495747153</v>
       </c>
       <c r="M599">
         <v>72.3</v>
@@ -28806,7 +28806,7 @@
         <v>51</v>
       </c>
       <c r="L600">
-        <v>0.3913410060913112</v>
+        <v>0.3913410060913111</v>
       </c>
       <c r="M600">
         <v>71.8</v>
@@ -28894,7 +28894,7 @@
         <v>57</v>
       </c>
       <c r="L602">
-        <v>0.3994063340877063</v>
+        <v>0.3994063340877062</v>
       </c>
       <c r="M602">
         <v>71.09999999999999</v>
@@ -28938,7 +28938,7 @@
         <v>38</v>
       </c>
       <c r="L603">
-        <v>0.4074465583140336</v>
+        <v>0.4074465583140335</v>
       </c>
       <c r="M603">
         <v>70.40000000000001</v>
@@ -28982,7 +28982,7 @@
         <v>25</v>
       </c>
       <c r="L604">
-        <v>0.4294466251134462</v>
+        <v>0.4294466251134461</v>
       </c>
       <c r="M604">
         <v>68.5</v>
@@ -29070,7 +29070,7 @@
         <v>44</v>
       </c>
       <c r="L606">
-        <v>0.4307719668634392</v>
+        <v>0.4307719668634391</v>
       </c>
       <c r="M606">
         <v>68.40000000000001</v>
@@ -29158,7 +29158,7 @@
         <v>32</v>
       </c>
       <c r="L608">
-        <v>0.4426673551836644</v>
+        <v>0.4426673551836643</v>
       </c>
       <c r="M608">
         <v>67.3</v>
@@ -29202,7 +29202,7 @@
         <v>33</v>
       </c>
       <c r="L609">
-        <v>0.4455000430090791</v>
+        <v>0.445500043009079</v>
       </c>
       <c r="M609">
         <v>67.09999999999999</v>
@@ -29246,7 +29246,7 @@
         <v>20</v>
       </c>
       <c r="L610">
-        <v>0.4506914493908503</v>
+        <v>0.4506914493908504</v>
       </c>
       <c r="M610">
         <v>66.59999999999999</v>
@@ -29466,7 +29466,7 @@
         <v>12</v>
       </c>
       <c r="L615">
-        <v>0.4645973876909517</v>
+        <v>0.4645973876909518</v>
       </c>
       <c r="M615">
         <v>65.40000000000001</v>
@@ -29510,7 +29510,7 @@
         <v>29</v>
       </c>
       <c r="L616">
-        <v>0.4665913547164852</v>
+        <v>0.4665913547164853</v>
       </c>
       <c r="M616">
         <v>65.2</v>
@@ -29598,7 +29598,7 @@
         <v>24</v>
       </c>
       <c r="L618">
-        <v>0.4719901317275148</v>
+        <v>0.4719901317275147</v>
       </c>
       <c r="M618">
         <v>64.7</v>
@@ -29642,7 +29642,7 @@
         <v>13</v>
       </c>
       <c r="L619">
-        <v>0.4785802485169127</v>
+        <v>0.4785802485169126</v>
       </c>
       <c r="M619">
         <v>64.2</v>
@@ -29950,7 +29950,7 @@
         <v>7</v>
       </c>
       <c r="L626">
-        <v>0.5116348158333914</v>
+        <v>0.5116348158333915</v>
       </c>
       <c r="M626">
         <v>61.3</v>
@@ -30082,7 +30082,7 @@
         <v>43</v>
       </c>
       <c r="L629">
-        <v>0.5360647817377521</v>
+        <v>0.536064781737752</v>
       </c>
       <c r="M629">
         <v>59.1</v>
@@ -30126,7 +30126,7 @@
         <v>48</v>
       </c>
       <c r="L630">
-        <v>0.539989451576208</v>
+        <v>0.5399894515762081</v>
       </c>
       <c r="M630">
         <v>58.8</v>
@@ -30258,7 +30258,7 @@
         <v>34</v>
       </c>
       <c r="L633">
-        <v>0.5508737731208408</v>
+        <v>0.550873773120841</v>
       </c>
       <c r="M633">
         <v>57.8</v>
@@ -30654,7 +30654,7 @@
         <v>64</v>
       </c>
       <c r="L642">
-        <v>0.7637005063489631</v>
+        <v>0.7637005063489632</v>
       </c>
       <c r="M642">
         <v>39.1</v>
@@ -30928,7 +30928,7 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>0.1403626871885737</v>
+        <v>0.1403626871885736</v>
       </c>
       <c r="M3">
         <v>98</v>
@@ -30972,7 +30972,7 @@
         <v>55</v>
       </c>
       <c r="L4">
-        <v>0.1474928229007858</v>
+        <v>0.1474928229007859</v>
       </c>
       <c r="M4">
         <v>96.7</v>
@@ -31060,7 +31060,7 @@
         <v>98</v>
       </c>
       <c r="L6">
-        <v>0.1496805428184261</v>
+        <v>0.149680542818426</v>
       </c>
       <c r="M6">
         <v>96.3</v>
@@ -31104,7 +31104,7 @@
         <v>58</v>
       </c>
       <c r="L7">
-        <v>0.1510480889393094</v>
+        <v>0.1510480889393095</v>
       </c>
       <c r="M7">
         <v>96.09999999999999</v>
@@ -31148,7 +31148,7 @@
         <v>38</v>
       </c>
       <c r="L8">
-        <v>0.1524535807715782</v>
+        <v>0.1524535807715783</v>
       </c>
       <c r="M8">
         <v>95.90000000000001</v>
@@ -31324,7 +31324,7 @@
         <v>66</v>
       </c>
       <c r="L12">
-        <v>0.1617839338873964</v>
+        <v>0.1617839338873965</v>
       </c>
       <c r="M12">
         <v>94.2</v>
@@ -31412,7 +31412,7 @@
         <v>115</v>
       </c>
       <c r="L14">
-        <v>0.06619144333400193</v>
+        <v>0.06619144333400194</v>
       </c>
       <c r="M14">
         <v>100</v>
@@ -31456,7 +31456,7 @@
         <v>136</v>
       </c>
       <c r="L15">
-        <v>0.06715442762708859</v>
+        <v>0.06715442762708856</v>
       </c>
       <c r="M15">
         <v>99.90000000000001</v>
@@ -31500,7 +31500,7 @@
         <v>127</v>
       </c>
       <c r="L16">
-        <v>0.07029108843014432</v>
+        <v>0.07029108843014437</v>
       </c>
       <c r="M16">
         <v>99.5</v>
@@ -31544,7 +31544,7 @@
         <v>107</v>
       </c>
       <c r="L17">
-        <v>0.07091316139324405</v>
+        <v>0.07091316139324408</v>
       </c>
       <c r="M17">
         <v>99.40000000000001</v>
@@ -31588,7 +31588,7 @@
         <v>109</v>
       </c>
       <c r="L18">
-        <v>0.07248601494447167</v>
+        <v>0.07248601494447171</v>
       </c>
       <c r="M18">
         <v>99.2</v>
@@ -31632,7 +31632,7 @@
         <v>123</v>
       </c>
       <c r="L19">
-        <v>0.07954104871917982</v>
+        <v>0.07954104871917984</v>
       </c>
       <c r="M19">
         <v>98.3</v>
@@ -31676,7 +31676,7 @@
         <v>142</v>
       </c>
       <c r="L20">
-        <v>0.08345345886506302</v>
+        <v>0.08345345886506304</v>
       </c>
       <c r="M20">
         <v>97.8</v>
@@ -31720,7 +31720,7 @@
         <v>147</v>
       </c>
       <c r="L21">
-        <v>0.0852218380005603</v>
+        <v>0.08522183800056025</v>
       </c>
       <c r="M21">
         <v>97.5</v>
@@ -31764,7 +31764,7 @@
         <v>103</v>
       </c>
       <c r="L22">
-        <v>0.08807377044332071</v>
+        <v>0.08807377044332075</v>
       </c>
       <c r="M22">
         <v>97.2</v>
@@ -31808,7 +31808,7 @@
         <v>94</v>
       </c>
       <c r="L23">
-        <v>0.08825008735098548</v>
+        <v>0.08825008735098551</v>
       </c>
       <c r="M23">
         <v>97.2</v>
@@ -31852,7 +31852,7 @@
         <v>130</v>
       </c>
       <c r="L24">
-        <v>0.08853929308511348</v>
+        <v>0.0885392930851135</v>
       </c>
       <c r="M24">
         <v>97.09999999999999</v>
@@ -31940,7 +31940,7 @@
         <v>93</v>
       </c>
       <c r="L26">
-        <v>0.09446266645596996</v>
+        <v>0.0944626664559699</v>
       </c>
       <c r="M26">
         <v>96.40000000000001</v>
@@ -31984,7 +31984,7 @@
         <v>95</v>
       </c>
       <c r="L27">
-        <v>0.09460288533901229</v>
+        <v>0.09460288533901234</v>
       </c>
       <c r="M27">
         <v>96.3</v>
@@ -32028,7 +32028,7 @@
         <v>104</v>
       </c>
       <c r="L28">
-        <v>0.09945727491143193</v>
+        <v>0.09945727491143191</v>
       </c>
       <c r="M28">
         <v>95.7</v>
@@ -32644,7 +32644,7 @@
         <v>28</v>
       </c>
       <c r="L42">
-        <v>0.07128055890117352</v>
+        <v>0.0712805589011736</v>
       </c>
       <c r="M42">
         <v>100</v>
@@ -32688,7 +32688,7 @@
         <v>26</v>
       </c>
       <c r="L43">
-        <v>0.07792670351053872</v>
+        <v>0.07792670351053879</v>
       </c>
       <c r="M43">
         <v>99.40000000000001</v>
@@ -32776,7 +32776,7 @@
         <v>39</v>
       </c>
       <c r="L45">
-        <v>0.1674395219602271</v>
+        <v>0.1674395219602272</v>
       </c>
       <c r="M45">
         <v>91.5</v>

</xml_diff>